<commit_message>
feat: update gender selection logic in registration process
</commit_message>
<xml_diff>
--- a/dataset/pendaftaran_sekolah.xlsx
+++ b/dataset/pendaftaran_sekolah.xlsx
@@ -580,11 +580,9 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.click: Error: strict mode violation: get_by_text("Pilih jenis kelamin", exact=True) resolved to 2 elements:
-    1) &lt;span data-v-cf5614bc="" class="line-clamp-2 text-gray-4"&gt;Pilih jenis kelamin&lt;/span&gt; aka get_by_text("Pilih jenis kelamin").first
-    2) &lt;span data-v-cf5614bc="" class="line-clamp-2 text-gray-4"&gt;Pilih jenis kelamin&lt;/span&gt; aka get_by_text("Pilih jenis kelamin").nth(1)
+          <t xml:space="preserve">FAILED: Locator.fill: Timeout 30000ms exceeded.
 Call log:
-  - waiting for get_by_text("Pilih jenis kelamin", exact=True)
+  - waiting for locator("input#nik\\ wali")
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat: update school registration dataset
</commit_message>
<xml_diff>
--- a/dataset/pendaftaran_sekolah.xlsx
+++ b/dataset/pendaftaran_sekolah.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="36000" windowHeight="20860" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3520" yWindow="-20980" windowWidth="28520" windowHeight="20860" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -455,8 +455,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
+  <dimension ref="A1:U32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="22.83203125" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -469,10 +469,12 @@
     <col width="10.83203125" customWidth="1" style="1" min="9" max="9"/>
     <col width="11.5" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="13.5" customWidth="1" min="12" max="12"/>
-    <col width="14.33203125" customWidth="1" min="13" max="13"/>
-    <col width="10.1640625" customWidth="1" min="14" max="14"/>
-    <col width="13.1640625" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="13.5" customWidth="1" min="12" max="13"/>
+    <col width="14.33203125" customWidth="1" min="14" max="14"/>
+    <col width="23.83203125" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="23.83203125" customWidth="1" min="16" max="16"/>
+    <col width="10.1640625" customWidth="1" min="17" max="17"/>
+    <col width="13.1640625" bestFit="1" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,30 +540,45 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>disabilitas</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>pekerjaan</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sekolah</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>jenjang_pendidikan</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
         <is>
           <t>prov</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>kab</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>kec</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>desa</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>domisili</t>
         </is>
@@ -575,20 +592,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bambang</t>
+          <t>Hasan Abdum</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.fill: Timeout 30000ms exceeded.
-Call log:
-  - waiting for locator("input#nik\\ wali")
-</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>1980-10-01</t>
+          <t>2019-01-26</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -629,30 +643,45 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Pegawai Swasta</t>
+          <t>Tidak memiliki disabilitas</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Pelajar</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>SD AL IRSYAD</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Kelas 1</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>Jawa Timur</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Kab. Situbondo</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Kendit</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Balung</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Jl. ABCD</t>
         </is>
@@ -661,32 +690,27 @@
     <row r="3" customFormat="1" s="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>3512345598191001</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Yuni</t>
+          <t>3512060209200001</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>KENZA SHAKIL AHMAD</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.click: Error: strict mode violation: get_by_text("Pilih jenis kelamin", exact=True) resolved to 2 elements:
-    1) &lt;span data-v-cf5614bc="" class="line-clamp-2 text-gray-4"&gt;Pilih jenis kelamin&lt;/span&gt; aka get_by_text("Pilih jenis kelamin").first
-    2) &lt;span data-v-cf5614bc="" class="line-clamp-2 text-gray-4"&gt;Pilih jenis kelamin&lt;/span&gt; aka get_by_text("Pilih jenis kelamin").nth(1)
-Call log:
-  - waiting for get_by_text("Pilih jenis kelamin", exact=True)
-</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>1990-12-01</t>
+          <t>2020-09-02</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Perempuan</t>
+          <t>Laki-laki</t>
         </is>
       </c>
       <c r="F3" s="1" t="n">
@@ -722,306 +746,180 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Pegawai Swasta</t>
+          <t>Tidak memiliki disabilitas</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>Pelajar</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>SD ISLAM AL ABROR</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Kelas 2</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>Jawa Timur</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Kab. Situbondo</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Kendit</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Balung</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Jl. ABCD</t>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Situbondo</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Patokan</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>KP TANAH ANYAR ALASMALANG RT 2 RW 5</t>
         </is>
       </c>
     </row>
     <row r="4" ht="17" customFormat="1" customHeight="1" s="3">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>3512345598191001</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Dwiki Aria</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>FAILED: name 'day_button' is not defined</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>2010-01-01</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>8123456789</v>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>3512052205820001</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>KUSYONO</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>1982-05-22</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>81234567890</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Belum Menikah</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Pegawai Swasta</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Jawa Timur</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Kab. Situbondo</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Kendit</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Balung</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Jl. ABCD</t>
-        </is>
-      </c>
+      <c r="A4" s="1" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>3512080107930050</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>BADRI FAUZI</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FAILED: Page.reload: Timeout 30000ms exceeded.
-Call log:
-  - waiting for navigation until "networkidle"
-    - navigated to "https://sehatindonesiaku.kemkes.go.id/ckg-pendaftaran-anak-sekolah"
-</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>1993-06-01</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>8123456789</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="inlineStr">
-        <is>
-          <t>3509116303960002</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>sri indriyani</t>
-        </is>
-      </c>
-      <c r="I5" s="1" t="inlineStr">
-        <is>
-          <t>1996-03-23</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>85231961508</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Menikah</t>
-        </is>
-      </c>
-      <c r="M5" s="1" t="inlineStr">
-        <is>
-          <t>ASN (Kantor Pemerintah)</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Jawa Timur</t>
-        </is>
-      </c>
-      <c r="O5" s="1" t="inlineStr">
-        <is>
-          <t>Kab. Situbondo</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Situbondo</t>
-        </is>
-      </c>
-      <c r="Q5" s="1" t="inlineStr">
-        <is>
-          <t>Kalibagor</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Kalibagor</t>
-        </is>
-      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="K5" s="1" t="n"/>
+      <c r="N5" s="1" t="n"/>
+      <c r="O5" s="1" t="n"/>
+      <c r="P5" s="1" t="n"/>
+      <c r="R5" s="1" t="n"/>
+      <c r="T5" s="1" t="n"/>
     </row>
     <row r="6">
       <c r="K6" s="1" t="n"/>
-      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n"/>
       <c r="O6" s="1" t="n"/>
-      <c r="Q6" s="1" t="n"/>
+      <c r="P6" s="1" t="n"/>
+      <c r="R6" s="1" t="n"/>
+      <c r="T6" s="1" t="n"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="C7" s="2" t="n"/>
       <c r="K7" s="1" t="n"/>
-      <c r="M7" s="1" t="n"/>
+      <c r="N7" s="1" t="n"/>
       <c r="O7" s="1" t="n"/>
-      <c r="Q7" s="1" t="n"/>
+      <c r="P7" s="1" t="n"/>
+      <c r="R7" s="1" t="n"/>
+      <c r="T7" s="1" t="n"/>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="C8" s="2" t="n"/>
       <c r="K8" s="1" t="n"/>
-      <c r="M8" s="1" t="n"/>
+      <c r="N8" s="1" t="n"/>
       <c r="O8" s="1" t="n"/>
-      <c r="Q8" s="1" t="n"/>
+      <c r="P8" s="1" t="n"/>
+      <c r="R8" s="1" t="n"/>
+      <c r="T8" s="1" t="n"/>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="C9" s="2" t="n"/>
       <c r="K9" s="1" t="n"/>
-      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="n"/>
       <c r="O9" s="1" t="n"/>
-      <c r="Q9" s="1" t="n"/>
+      <c r="P9" s="1" t="n"/>
+      <c r="R9" s="1" t="n"/>
+      <c r="T9" s="1" t="n"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="C10" s="2" t="n"/>
       <c r="K10" s="1" t="n"/>
-      <c r="M10" s="1" t="n"/>
+      <c r="N10" s="1" t="n"/>
+      <c r="O10" s="1" t="n"/>
+      <c r="P10" s="1" t="n"/>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="C11" s="2" t="n"/>
       <c r="K11" s="1" t="n"/>
-      <c r="M11" s="1" t="n"/>
+      <c r="N11" s="1" t="n"/>
       <c r="O11" s="1" t="n"/>
-      <c r="Q11" s="1" t="n"/>
+      <c r="P11" s="1" t="n"/>
+      <c r="R11" s="1" t="n"/>
+      <c r="T11" s="1" t="n"/>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="C12" s="2" t="n"/>
       <c r="K12" s="1" t="n"/>
-      <c r="M12" s="1" t="n"/>
+      <c r="N12" s="1" t="n"/>
       <c r="O12" s="1" t="n"/>
-      <c r="Q12" s="1" t="n"/>
+      <c r="P12" s="1" t="n"/>
+      <c r="R12" s="1" t="n"/>
+      <c r="T12" s="1" t="n"/>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="C13" s="2" t="n"/>
       <c r="K13" s="1" t="n"/>
-      <c r="M13" s="1" t="n"/>
+      <c r="N13" s="1" t="n"/>
       <c r="O13" s="1" t="n"/>
-      <c r="Q13" s="1" t="n"/>
+      <c r="P13" s="1" t="n"/>
+      <c r="R13" s="1" t="n"/>
+      <c r="T13" s="1" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="C14" s="2" t="n"/>
       <c r="K14" s="1" t="n"/>
-      <c r="M14" s="1" t="n"/>
+      <c r="N14" s="1" t="n"/>
       <c r="O14" s="1" t="n"/>
-      <c r="Q14" s="1" t="n"/>
+      <c r="P14" s="1" t="n"/>
+      <c r="R14" s="1" t="n"/>
+      <c r="T14" s="1" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="C15" s="2" t="n"/>
       <c r="K15" s="1" t="n"/>
-      <c r="M15" s="1" t="n"/>
+      <c r="N15" s="1" t="n"/>
       <c r="O15" s="1" t="n"/>
-      <c r="Q15" s="1" t="n"/>
+      <c r="P15" s="1" t="n"/>
+      <c r="R15" s="1" t="n"/>
+      <c r="T15" s="1" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="C16" s="2" t="n"/>
       <c r="K16" s="1" t="n"/>
-      <c r="M16" s="1" t="n"/>
+      <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="n"/>
-      <c r="Q16" s="1" t="n"/>
+      <c r="P16" s="1" t="n"/>
+      <c r="R16" s="1" t="n"/>
+      <c r="T16" s="1" t="n"/>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="C17" s="2" t="n"/>
       <c r="K17" s="1" t="n"/>
-      <c r="M17" s="1" t="n"/>
+      <c r="N17" s="1" t="n"/>
       <c r="O17" s="1" t="n"/>
-      <c r="Q17" s="1" t="n"/>
+      <c r="P17" s="1" t="n"/>
+      <c r="R17" s="1" t="n"/>
+      <c r="T17" s="1" t="n"/>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="C18" s="2" t="n"/>
       <c r="K18" s="1" t="n"/>
-      <c r="M18" s="1" t="n"/>
+      <c r="N18" s="1" t="n"/>
       <c r="O18" s="1" t="n"/>
-      <c r="Q18" s="1" t="n"/>
+      <c r="P18" s="1" t="n"/>
+      <c r="R18" s="1" t="n"/>
+      <c r="T18" s="1" t="n"/>
     </row>
     <row r="19"/>
     <row r="20"/>
@@ -1049,6 +947,9 @@
       <c r="J32" s="1" t="n"/>
       <c r="L32" s="1" t="n"/>
       <c r="M32" s="1" t="n"/>
+      <c r="N32" s="1" t="n"/>
+      <c r="O32" s="1" t="n"/>
+      <c r="P32" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>